<commit_message>
updates with mixing depth at 200 kyr
</commit_message>
<xml_diff>
--- a/blueIceData.xlsx
+++ b/blueIceData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jesst/Library/CloudStorage/Dropbox/blueIce/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0502B85-75FA-A04F-AA95-5E05D70AD64F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{772B8B35-F431-A346-8DB3-669744C7AC42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18260" yWindow="10140" windowWidth="29380" windowHeight="15140" xr2:uid="{E7B7DD3A-D12D-CA45-8402-C1170DE88CFD}"/>
+    <workbookView xWindow="10320" yWindow="3120" windowWidth="29380" windowHeight="15140" xr2:uid="{E7B7DD3A-D12D-CA45-8402-C1170DE88CFD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>